<commit_message>
data uptaded to march 2026 and inflation data added
</commit_message>
<xml_diff>
--- a/data/original/banco_republica/unemployment/unemployment.xlsx
+++ b/data/original/banco_republica/unemployment/unemployment.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="567">
   <si>
     <t>Fecha</t>
   </si>
@@ -1664,10 +1664,19 @@
     <t>31/01/2026</t>
   </si>
   <si>
+    <t>28/02/2026</t>
+  </si>
+  <si>
+    <t>31/03/2026</t>
+  </si>
+  <si>
+    <t>8,79</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Descargado de sistema del Banco de la República martes, 3 de marzo de 2026 8:03:08 p. m.</t>
+    <t>Descargado de sistema del Banco de la República martes, 5 de mayo de 2026 1:20:17 p. m.</t>
   </si>
   <si>
     <t>Nombre de la serie</t>
@@ -2091,7 +2100,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B306"/>
+  <dimension ref="A1:B308"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -4522,19 +4531,35 @@
         <v>157</v>
       </c>
     </row>
-    <row r="304" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
         <v>550</v>
       </c>
-    </row>
-    <row r="305" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B304" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>550</v>
+        <v>551</v>
+      </c>
+      <c r="B305" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="306" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>551</v>
+        <v>553</v>
+      </c>
+    </row>
+    <row r="307" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A307" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="308" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A308" t="s">
+        <v>554</v>
       </c>
     </row>
   </sheetData>
@@ -4557,48 +4582,48 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
general fixes in population and cpi, as well as some generalizations
</commit_message>
<xml_diff>
--- a/data/original/banco_republica/unemployment/unemployment.xlsx
+++ b/data/original/banco_republica/unemployment/unemployment.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="567">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="568">
   <si>
     <t>Fecha</t>
   </si>
@@ -1673,10 +1673,13 @@
     <t>8,79</t>
   </si>
   <si>
+    <t>30/04/2026</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Descargado de sistema del Banco de la República martes, 5 de mayo de 2026 1:20:17 p. m.</t>
+    <t>Descargado de sistema del Banco de la República lunes, 1 de junio de 2026 8:18:03 p. m.</t>
   </si>
   <si>
     <t>Nombre de la serie</t>
@@ -2100,7 +2103,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B308"/>
+  <dimension ref="A1:B309"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -4547,19 +4550,27 @@
         <v>552</v>
       </c>
     </row>
-    <row r="306" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
         <v>553</v>
       </c>
+      <c r="B306" t="s">
+        <v>534</v>
+      </c>
     </row>
     <row r="307" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="308" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
         <v>554</v>
+      </c>
+    </row>
+    <row r="309" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A309" t="s">
+        <v>555</v>
       </c>
     </row>
   </sheetData>
@@ -4582,48 +4593,48 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
   </sheetData>

</xml_diff>